<commit_message>
Adicionado gráficos e dados de detecção por métodos estatísticos
</commit_message>
<xml_diff>
--- a/experiment_results/combined_sweep/rtt_bursts_S1_atk10pct_wu300000.xlsx
+++ b/experiment_results/combined_sweep/rtt_bursts_S1_atk10pct_wu300000.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -548,12 +548,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -605,12 +605,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>21393</t>
+          <t>11703</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -662,12 +662,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>22923</t>
+          <t>11220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>0.68</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>24587</t>
+          <t>13367</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.14</t>
+          <t>0.41</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>38509</t>
+          <t>25142</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.64</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79993</t>
+          <t>54851</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>117818</t>
+          <t>62966</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -947,12 +947,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.63</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>128894</t>
+          <t>65927</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>0.64</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>130212</t>
+          <t>64285</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>126897</t>
+          <t>62612</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>126227</t>
+          <t>63615</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.71</t>
+          <t>0.65</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>127979</t>
+          <t>64363</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1232,12 +1232,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>133733</t>
+          <t>69370</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1289,12 +1289,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>140797</t>
+          <t>71427</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1346,12 +1346,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>139619</t>
+          <t>68192</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1403,12 +1403,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>133266</t>
+          <t>65074</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1460,12 +1460,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>130147</t>
+          <t>65074</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">

</xml_diff>